<commit_message>
Daily scans — 14-May-2026 20:51 — 18 file(s)
</commit_message>
<xml_diff>
--- a/50EMA_Shakeout_v1_2026-05-14.xlsx
+++ b/50EMA_Shakeout_v1_2026-05-14.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📺 TV Watchlist" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'🔥 Reclaimed Today'!$A$1:$P$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'🎯 Reclaimed 1-3 Days'!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'🔥 Reclaimed Today'!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'🎯 Reclaimed 1-3 Days'!$A$1:$P$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -184,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -213,9 +213,6 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -225,19 +222,28 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -633,15 +639,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -739,26 +745,26 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>NATIONALUM</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>3.12</v>
+        <v>3.06</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>370.69</v>
+        <v>412.92</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>408.25</v>
+        <v>1303.6</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>397.92</v>
+        <v>1275.08</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>320.05</v>
+        <v>1260.25</v>
       </c>
       <c r="H2" s="6" t="n">
         <v>0</v>
@@ -767,10 +773,10 @@
         <v>2</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>2.58</v>
+        <v>3</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>0.97</v>
+        <v>0.9</v>
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
@@ -791,359 +797,11 @@
         <v>9.039999999999999</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>9.039999999999999</v>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>ROSSTECH</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>98</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>7.33</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>12.93</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>875.8</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>844.87</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>699.15</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="5" t="n">
-        <v>2.46</v>
-      </c>
-      <c r="K3" s="10" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="L3" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M3" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N3" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="n">
-        <v>21.25</v>
-      </c>
-      <c r="P3" s="4" t="n">
-        <v>21.25</v>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>GPIL</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>97</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>3.22</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>85.28</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>290</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>283.84</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>255.71</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="5" t="n">
-        <v>2.34</v>
-      </c>
-      <c r="K4" s="7" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="L4" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="M4" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N4" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>163.79</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>7.84</v>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>TMB</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>97</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>61.25</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>681.6</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>665.89</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>570.83</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" s="5" t="n">
-        <v>2.36</v>
-      </c>
-      <c r="K5" s="7" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="L5" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="M5" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N5" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O5" s="4" t="n">
-        <v>12.97</v>
-      </c>
-      <c r="P5" s="4" t="n">
-        <v>12.97</v>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>HEG</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>93</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>4.44</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>170.43</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>604.3</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>584.87</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>544.13</v>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="5" t="n">
-        <v>3.76</v>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="L6" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="M6" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N6" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>14.18</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>14.18</v>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>PREMEXPLN</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>80</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>4.82</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>22.09</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>542</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>505</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>507.77</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="5" t="n">
-        <v>8.710000000000001</v>
-      </c>
-      <c r="K7" s="10" t="n">
-        <v>2.42</v>
-      </c>
-      <c r="L7" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M7" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N7" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O7" s="4" t="n">
-        <v>67.68000000000001</v>
-      </c>
-      <c r="P7" s="4" t="n">
-        <v>26.2</v>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>PNGJL</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>78</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>21.49</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>631.95</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>628</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>608</v>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="5" t="n">
-        <v>4.29</v>
-      </c>
-      <c r="K8" s="10" t="n">
-        <v>2.09</v>
-      </c>
-      <c r="L8" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M8" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N8" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>34.19</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>16.53</v>
+        <v>5.84</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P8"/>
+  <autoFilter ref="A1:P2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1155,15 +813,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -1259,65 +917,587 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>ROSSTECH</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="n">
+        <v>98</v>
+      </c>
+      <c r="C2" s="12" t="n">
+        <v>7.27</v>
+      </c>
+      <c r="D2" s="13" t="n">
+        <v>13.09</v>
+      </c>
+      <c r="E2" s="12" t="n">
+        <v>932.75</v>
+      </c>
+      <c r="F2" s="12" t="n">
+        <v>848.3200000000001</v>
+      </c>
+      <c r="G2" s="12" t="n">
+        <v>701.48</v>
+      </c>
+      <c r="H2" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="13" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="K2" s="14" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M2" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N2" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O2" s="12" t="n">
+        <v>13.85</v>
+      </c>
+      <c r="P2" s="12" t="n">
+        <v>13.85</v>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>NATIONALUM</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>98</v>
+      </c>
+      <c r="C3" s="12" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D3" s="13" t="n">
+        <v>370.54</v>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>416.45</v>
+      </c>
+      <c r="F3" s="12" t="n">
+        <v>398.65</v>
+      </c>
+      <c r="G3" s="12" t="n">
+        <v>321.01</v>
+      </c>
+      <c r="H3" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" s="13" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="K3" s="17" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L3" s="18" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="M3" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N3" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O3" s="12" t="n">
+        <v>6.89</v>
+      </c>
+      <c r="P3" s="12" t="n">
+        <v>6.89</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>SAKAR</t>
         </is>
       </c>
-      <c r="B2" s="12" t="n">
+      <c r="B4" s="11" t="n">
         <v>98</v>
       </c>
-      <c r="C2" s="13" t="n">
-        <v>6.75</v>
-      </c>
-      <c r="D2" s="14" t="n">
-        <v>8.279999999999999</v>
-      </c>
-      <c r="E2" s="13" t="n">
-        <v>599.45</v>
-      </c>
-      <c r="F2" s="13" t="n">
-        <v>560</v>
-      </c>
-      <c r="G2" s="13" t="n">
-        <v>452.39</v>
-      </c>
-      <c r="H2" s="12" t="n">
+      <c r="C4" s="12" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>599.8</v>
+      </c>
+      <c r="F4" s="12" t="n">
+        <v>561.5599999999999</v>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>453.85</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" s="13" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>6.88</v>
+      </c>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N4" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O4" s="12" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="P4" s="12" t="n">
+        <v>10.36</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>GPIL</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>97</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>78.23</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>289.25</v>
+      </c>
+      <c r="F5" s="12" t="n">
+        <v>284.05</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>256.04</v>
+      </c>
+      <c r="H5" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="J2" s="16" t="n">
-        <v>7.28</v>
-      </c>
-      <c r="K2" s="17" t="n">
-        <v>6.88</v>
-      </c>
-      <c r="L2" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="M2" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="N2" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="O2" s="13" t="n">
-        <v>10.43</v>
-      </c>
-      <c r="P2" s="13" t="n">
-        <v>10.43</v>
+      <c r="I5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="13" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="K5" s="17" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="L5" s="18" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O5" s="12" t="n">
+        <v>164.48</v>
+      </c>
+      <c r="P5" s="12" t="n">
+        <v>8.119999999999999</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>TMB</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>61.16</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>666.35</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>665.91</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>571.78</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="13" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="K6" s="17" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="M6" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N6" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O6" s="12" t="n">
+        <v>15.55</v>
+      </c>
+      <c r="P6" s="12" t="n">
+        <v>15.55</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>HEG</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>94</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>166.2</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>617.65</v>
+      </c>
+      <c r="F7" s="12" t="n">
+        <v>586.15</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>544.87</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="13" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="K7" s="17" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L7" s="18" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O7" s="12" t="n">
+        <v>11.71</v>
+      </c>
+      <c r="P7" s="12" t="n">
+        <v>11.71</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>CARERATING</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>91</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>1735.7</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>1605.73</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>1569.4</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="K8" s="17" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="M8" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N8" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O8" s="12" t="n">
+        <v>13.15</v>
+      </c>
+      <c r="P8" s="12" t="n">
+        <v>13.15</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>PNGJL</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>78</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>637.65</v>
+      </c>
+      <c r="F9" s="12" t="n">
+        <v>628.38</v>
+      </c>
+      <c r="G9" s="12" t="n">
+        <v>608.3</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="13" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="L9" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O9" s="12" t="n">
+        <v>32.99</v>
+      </c>
+      <c r="P9" s="12" t="n">
+        <v>15.49</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>PREMEXPLN</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>78</v>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>23.91</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>544.1</v>
+      </c>
+      <c r="F10" s="12" t="n">
+        <v>506.53</v>
+      </c>
+      <c r="G10" s="12" t="n">
+        <v>508.13</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="13" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="K10" s="14" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="L10" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M10" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N10" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O10" s="12" t="n">
+        <v>67.03</v>
+      </c>
+      <c r="P10" s="12" t="n">
+        <v>25.71</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>WELENT</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>76</v>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>22.34</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>518.4</v>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>491.13</v>
+      </c>
+      <c r="G11" s="12" t="n">
+        <v>495.21</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="13" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="K11" s="17" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="L11" s="18" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="O11" s="12" t="n">
+        <v>26.35</v>
+      </c>
+      <c r="P11" s="12" t="n">
+        <v>11.88</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P2"/>
+  <autoFilter ref="A1:P11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1337,75 +1517,75 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
-        <is>
-          <t>📺  50 EMA Shakeout Scanner  —  13-May-2026  23:29 IST</t>
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>📺  50 EMA Shakeout Scanner  —  14-May-2026  20:08 IST</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">  ✂  Click orange cell → Ctrl+C → TradingView → Watchlist → (...) → Import List → Paste</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🔥 Reclaimed Today   —   7 stocks</t>
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🔥 Reclaimed Today   —   1 stocks</t>
         </is>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  7 symbols</t>
-        </is>
-      </c>
-      <c r="B4" s="23" t="inlineStr">
-        <is>
-          <t>NSE:NATIONALUM,NSE:ROSSTECH,NSE:GPIL,NSE:TMB,NSE:HEG,NSE:PREMEXPLN,NSE:PNGJL</t>
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1 symbols</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>NSE:DRREDDY</t>
         </is>
       </c>
     </row>
     <row r="5" ht="6" customHeight="1"/>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🎯 Reclaimed 1-3 Days   —   1 stocks</t>
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🎯 Reclaimed 1-3 Days   —   10 stocks</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1 symbols</t>
-        </is>
-      </c>
-      <c r="B7" s="23" t="inlineStr">
-        <is>
-          <t>NSE:SAKAR</t>
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  10 symbols</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>NSE:ROSSTECH,NSE:NATIONALUM,NSE:SAKAR,NSE:GPIL,NSE:TMB,NSE:HEG,NSE:CARERATING,NSE:PNGJL,NSE:PREMEXPLN,NSE:WELENT</t>
         </is>
       </c>
     </row>
     <row r="8" ht="6" customHeight="1"/>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  📊 All Combined   —   8 stocks</t>
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  📊 All Combined   —   11 stocks</t>
         </is>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  8 symbols</t>
-        </is>
-      </c>
-      <c r="B10" s="23" t="inlineStr">
-        <is>
-          <t>NSE:NATIONALUM,NSE:ROSSTECH,NSE:GPIL,NSE:TMB,NSE:HEG,NSE:PREMEXPLN,NSE:PNGJL,NSE:SAKAR</t>
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  11 symbols</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>NSE:DRREDDY,NSE:ROSSTECH,NSE:NATIONALUM,NSE:SAKAR,NSE:GPIL,NSE:TMB,NSE:HEG,NSE:CARERATING,NSE:PNGJL,NSE:PREMEXPLN,NSE:WELENT</t>
         </is>
       </c>
     </row>

</xml_diff>